<commit_message>
Adding minimal FSOE packets to PDO map
</commit_message>
<xml_diff>
--- a/Core0-freertos/src/EtherCAT/SSC/SSC-AM2612.xlsx
+++ b/Core0-freertos/src/EtherCAT/SSC/SSC-AM2612.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Profile" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Profile!$B$1:$P$72</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Profile!$B$10:$P$73</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">Profile!$B$1:$P$82</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Profile!$B$10:$P$83</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="100">
   <si>
     <t xml:space="preserve">Device Profile:</t>
   </si>
@@ -363,6 +363,30 @@
     <t xml:space="preserve">Complex_Double</t>
   </si>
   <si>
+    <t xml:space="preserve">0x6100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FSOE_Tx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fsoeStatus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">safeInputs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UINT16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">connectionId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fsoeCRC</t>
+  </si>
+  <si>
     <t xml:space="preserve">//0x7nnx</t>
   </si>
   <si>
@@ -375,9 +399,6 @@
     <t xml:space="preserve">Single_Byte_Rx</t>
   </si>
   <si>
-    <t xml:space="preserve">rw</t>
-  </si>
-  <si>
     <t xml:space="preserve">rx</t>
   </si>
   <si>
@@ -399,6 +420,18 @@
     <t xml:space="preserve">Complex_Rx</t>
   </si>
   <si>
+    <t xml:space="preserve">0x7100</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FSOE_Rx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fsoeCommand</t>
+  </si>
+  <si>
+    <t xml:space="preserve">safeOutputs</t>
+  </si>
+  <si>
     <t xml:space="preserve">//0x8nnx</t>
   </si>
   <si>
@@ -427,9 +460,6 @@
   </si>
   <si>
     <t xml:space="preserve">m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">UINT16</t>
   </si>
   <si>
     <t xml:space="preserve">Index distance </t>
@@ -944,7 +974,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:T922"/>
+  <dimension ref="A1:T932"/>
   <sheetFormatPr defaultColWidth="10.71484375" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="1" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="3.86"/>
@@ -1857,8 +1887,8 @@
       <c r="M43" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="N43" s="0"/>
-      <c r="O43" s="0"/>
+      <c r="N43" s="21"/>
+      <c r="O43" s="21"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="2"/>
@@ -1975,46 +2005,48 @@
       <c r="S47" s="1"/>
       <c r="T47" s="1"/>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="13"/>
-      <c r="B48" s="14" t="s">
+    <row r="48" s="15" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="2"/>
+      <c r="B48" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C48" s="14" t="s">
+      <c r="C48" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D48" s="19"/>
+      <c r="E48" s="13"/>
+      <c r="F48" s="13" t="s">
         <v>65</v>
       </c>
-      <c r="D48" s="14"/>
-      <c r="E48" s="14"/>
-      <c r="F48" s="14"/>
-      <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
-      <c r="I48" s="14"/>
-      <c r="J48" s="14"/>
-      <c r="K48" s="14"/>
-      <c r="L48" s="14"/>
-      <c r="M48" s="14"/>
-      <c r="N48" s="14"/>
-      <c r="O48" s="14"/>
-      <c r="P48" s="14"/>
-      <c r="Q48" s="15"/>
-      <c r="R48" s="15"/>
-      <c r="S48" s="15"/>
-      <c r="T48" s="15"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="G48" s="13"/>
+      <c r="H48" s="13"/>
+      <c r="I48" s="13"/>
+      <c r="J48" s="2"/>
+      <c r="K48" s="2"/>
+      <c r="L48" s="2"/>
+      <c r="M48" s="2"/>
+      <c r="N48" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O48" s="1"/>
+      <c r="P48" s="1"/>
+      <c r="Q48" s="1"/>
+      <c r="R48" s="1"/>
+      <c r="S48" s="1"/>
+      <c r="T48" s="1"/>
+    </row>
+    <row r="49" s="15" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2"/>
-      <c r="B49" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D49" s="19"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="19" t="n">
+        <v>1</v>
+      </c>
       <c r="E49" s="13" t="s">
         <v>41</v>
       </c>
       <c r="F49" s="13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G49" s="13" t="s">
         <v>4</v>
@@ -2024,44 +2056,66 @@
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
       <c r="L49" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M49" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="N49" s="1"/>
+      <c r="O49" s="1"/>
+      <c r="P49" s="1"/>
+      <c r="Q49" s="1"/>
+      <c r="R49" s="1"/>
+      <c r="S49" s="1"/>
+      <c r="T49" s="1"/>
+    </row>
+    <row r="50" s="15" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="2"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F50" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="M49" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D50" s="19"/>
-      <c r="E50" s="13"/>
-      <c r="F50" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="G50" s="13"/>
+      <c r="G50" s="13" t="s">
+        <v>4</v>
+      </c>
       <c r="H50" s="13"/>
       <c r="I50" s="13"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
-      <c r="L50" s="2"/>
-      <c r="M50" s="2"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L50" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M50" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="N50" s="1"/>
+      <c r="O50" s="1"/>
+      <c r="P50" s="1"/>
+      <c r="Q50" s="1"/>
+      <c r="R50" s="1"/>
+      <c r="S50" s="1"/>
+      <c r="T50" s="1"/>
+    </row>
+    <row r="51" s="15" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E51" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="F51" s="13"/>
+        <v>69</v>
+      </c>
+      <c r="F51" s="13" t="s">
+        <v>70</v>
+      </c>
       <c r="G51" s="13" t="s">
         <v>4</v>
       </c>
@@ -2070,25 +2124,32 @@
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
       <c r="L51" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M51" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="N51" s="0"/>
-      <c r="O51" s="0"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>44</v>
+      </c>
+      <c r="N51" s="1"/>
+      <c r="O51" s="1"/>
+      <c r="P51" s="1"/>
+      <c r="Q51" s="1"/>
+      <c r="R51" s="1"/>
+      <c r="S51" s="1"/>
+      <c r="T51" s="1"/>
+    </row>
+    <row r="52" s="15" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
       <c r="D52" s="19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="F52" s="13"/>
+        <v>69</v>
+      </c>
+      <c r="F52" s="13" t="s">
+        <v>71</v>
+      </c>
       <c r="G52" s="13" t="s">
         <v>4</v>
       </c>
@@ -2097,51 +2158,59 @@
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
       <c r="L52" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M52" s="2" t="s">
-        <v>69</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="N52" s="1"/>
+      <c r="O52" s="1"/>
+      <c r="P52" s="1"/>
+      <c r="Q52" s="1"/>
+      <c r="R52" s="1"/>
+      <c r="S52" s="1"/>
+      <c r="T52" s="1"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="2"/>
-      <c r="D53" s="19" t="n">
-        <v>3</v>
-      </c>
-      <c r="E53" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="F53" s="13"/>
-      <c r="G53" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="H53" s="13"/>
-      <c r="I53" s="13"/>
-      <c r="J53" s="2"/>
-      <c r="K53" s="2"/>
-      <c r="L53" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="M53" s="2" t="s">
-        <v>69</v>
-      </c>
+      <c r="A53" s="13"/>
+      <c r="B53" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C53" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="D53" s="14"/>
+      <c r="E53" s="14"/>
+      <c r="F53" s="14"/>
+      <c r="G53" s="14"/>
+      <c r="H53" s="14"/>
+      <c r="I53" s="14"/>
+      <c r="J53" s="14"/>
+      <c r="K53" s="14"/>
+      <c r="L53" s="14"/>
+      <c r="M53" s="14"/>
+      <c r="N53" s="14"/>
+      <c r="O53" s="14"/>
+      <c r="P53" s="14"/>
+      <c r="Q53" s="15"/>
+      <c r="R53" s="15"/>
+      <c r="S53" s="15"/>
+      <c r="T53" s="15"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="2"/>
       <c r="B54" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C54" s="2" t="s">
         <v>40</v>
       </c>
       <c r="D54" s="19"/>
       <c r="E54" s="13" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="F54" s="13" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G54" s="13" t="s">
         <v>4</v>
@@ -2151,24 +2220,24 @@
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
       <c r="L54" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M54" s="2" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="2"/>
       <c r="B55" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="D55" s="19"/>
       <c r="E55" s="13"/>
       <c r="F55" s="13" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="G55" s="13"/>
       <c r="H55" s="13"/>
@@ -2177,9 +2246,6 @@
       <c r="K55" s="2"/>
       <c r="L55" s="2"/>
       <c r="M55" s="2"/>
-      <c r="N55" s="1" t="s">
-        <v>55</v>
-      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="2"/>
@@ -2191,9 +2257,7 @@
       <c r="E56" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="F56" s="13" t="s">
-        <v>56</v>
-      </c>
+      <c r="F56" s="13"/>
       <c r="G56" s="13" t="s">
         <v>4</v>
       </c>
@@ -2202,11 +2266,13 @@
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
       <c r="L56" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M56" s="2" t="s">
-        <v>69</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="N56" s="21"/>
+      <c r="O56" s="21"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2"/>
@@ -2216,11 +2282,9 @@
         <v>2</v>
       </c>
       <c r="E57" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="F57" s="13" t="s">
-        <v>57</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="F57" s="13"/>
       <c r="G57" s="13" t="s">
         <v>4</v>
       </c>
@@ -2229,10 +2293,10 @@
       <c r="J57" s="2"/>
       <c r="K57" s="2"/>
       <c r="L57" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M57" s="2" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2243,11 +2307,9 @@
         <v>3</v>
       </c>
       <c r="E58" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="F58" s="13" t="s">
-        <v>59</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="F58" s="13"/>
       <c r="G58" s="13" t="s">
         <v>4</v>
       </c>
@@ -2256,24 +2318,26 @@
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
       <c r="L58" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M58" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="59" s="15" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="2"/>
-      <c r="D59" s="19" t="n">
-        <v>4</v>
-      </c>
+      <c r="B59" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D59" s="19"/>
       <c r="E59" s="13" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F59" s="13" t="s">
-        <v>61</v>
+        <v>80</v>
       </c>
       <c r="G59" s="13" t="s">
         <v>4</v>
@@ -2283,164 +2347,191 @@
       <c r="J59" s="2"/>
       <c r="K59" s="2"/>
       <c r="L59" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M59" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="N59" s="1"/>
-      <c r="O59" s="1"/>
-      <c r="P59" s="1"/>
-      <c r="Q59" s="1"/>
-      <c r="R59" s="1"/>
-      <c r="S59" s="1"/>
-      <c r="T59" s="1"/>
+        <v>76</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="2"/>
-      <c r="D60" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="E60" s="13" t="s">
-        <v>62</v>
-      </c>
+      <c r="B60" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D60" s="19"/>
+      <c r="E60" s="13"/>
       <c r="F60" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="G60" s="13" t="s">
-        <v>4</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="G60" s="13"/>
       <c r="H60" s="13"/>
       <c r="I60" s="13"/>
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
-      <c r="L60" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="M60" s="2" t="s">
-        <v>69</v>
+      <c r="L60" s="2"/>
+      <c r="M60" s="2"/>
+      <c r="N60" s="1" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="13"/>
-      <c r="B61" s="14" t="s">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="F61" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G61" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="H61" s="13"/>
+      <c r="I61" s="13"/>
+      <c r="J61" s="2"/>
+      <c r="K61" s="2"/>
+      <c r="L61" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M61" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C61" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="D61" s="14"/>
-      <c r="E61" s="14"/>
-      <c r="F61" s="14"/>
-      <c r="G61" s="14"/>
-      <c r="H61" s="14"/>
-      <c r="I61" s="14"/>
-      <c r="J61" s="14"/>
-      <c r="K61" s="14"/>
-      <c r="L61" s="14"/>
-      <c r="M61" s="14"/>
-      <c r="N61" s="14"/>
-      <c r="O61" s="14"/>
-      <c r="P61" s="14"/>
-      <c r="Q61" s="15"/>
-      <c r="R61" s="15"/>
-      <c r="S61" s="15"/>
-      <c r="T61" s="15"/>
-    </row>
-    <row r="62" s="15" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="2"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
-      <c r="D62" s="19"/>
-      <c r="E62" s="13"/>
-      <c r="F62" s="13"/>
-      <c r="G62" s="13"/>
+      <c r="D62" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E62" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F62" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="G62" s="13" t="s">
+        <v>4</v>
+      </c>
       <c r="H62" s="13"/>
       <c r="I62" s="13"/>
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
-      <c r="L62" s="2"/>
-      <c r="M62" s="2"/>
-      <c r="N62" s="1"/>
-      <c r="O62" s="1"/>
-      <c r="P62" s="1"/>
-      <c r="Q62" s="1"/>
-      <c r="R62" s="1"/>
-      <c r="S62" s="1"/>
-      <c r="T62" s="1"/>
+      <c r="L62" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M62" s="2" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="2"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
-      <c r="D63" s="19"/>
-      <c r="E63" s="13"/>
-      <c r="F63" s="13"/>
-      <c r="G63" s="13"/>
+      <c r="D63" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E63" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="F63" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="G63" s="13" t="s">
+        <v>4</v>
+      </c>
       <c r="H63" s="13"/>
       <c r="I63" s="13"/>
       <c r="J63" s="2"/>
       <c r="K63" s="2"/>
-      <c r="L63" s="2"/>
-      <c r="M63" s="2"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="13"/>
-      <c r="B64" s="14" t="s">
-        <v>78</v>
-      </c>
-      <c r="C64" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="D64" s="14"/>
-      <c r="E64" s="14"/>
-      <c r="F64" s="14"/>
-      <c r="G64" s="14"/>
-      <c r="H64" s="14"/>
-      <c r="I64" s="14"/>
-      <c r="J64" s="14"/>
-      <c r="K64" s="14"/>
-      <c r="L64" s="14"/>
-      <c r="M64" s="14"/>
-      <c r="N64" s="14"/>
-      <c r="O64" s="14"/>
-      <c r="P64" s="14"/>
-      <c r="Q64" s="15"/>
-      <c r="R64" s="15"/>
-      <c r="S64" s="15"/>
-      <c r="T64" s="15"/>
-    </row>
-    <row r="65" s="15" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L63" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M63" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="64" s="15" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="2"/>
+      <c r="B64" s="2"/>
+      <c r="C64" s="2"/>
+      <c r="D64" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E64" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="F64" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="G64" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="H64" s="13"/>
+      <c r="I64" s="13"/>
+      <c r="J64" s="2"/>
+      <c r="K64" s="2"/>
+      <c r="L64" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M64" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="N64" s="1"/>
+      <c r="O64" s="1"/>
+      <c r="P64" s="1"/>
+      <c r="Q64" s="1"/>
+      <c r="R64" s="1"/>
+      <c r="S64" s="1"/>
+      <c r="T64" s="1"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="2"/>
       <c r="B65" s="2"/>
       <c r="C65" s="2"/>
-      <c r="D65" s="19"/>
-      <c r="E65" s="13"/>
-      <c r="F65" s="13"/>
-      <c r="G65" s="13"/>
+      <c r="D65" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="E65" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="F65" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="G65" s="13" t="s">
+        <v>4</v>
+      </c>
       <c r="H65" s="13"/>
       <c r="I65" s="13"/>
       <c r="J65" s="2"/>
       <c r="K65" s="2"/>
-      <c r="L65" s="2"/>
-      <c r="M65" s="2"/>
-      <c r="N65" s="1"/>
-      <c r="O65" s="1"/>
-      <c r="P65" s="1"/>
-      <c r="Q65" s="1"/>
-      <c r="R65" s="1"/>
-      <c r="S65" s="1"/>
-      <c r="T65" s="1"/>
+      <c r="L65" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M65" s="2" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="2"/>
+      <c r="B66" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="D66" s="19"/>
       <c r="E66" s="13"/>
-      <c r="F66" s="13"/>
+      <c r="F66" s="13" t="s">
+        <v>84</v>
+      </c>
       <c r="G66" s="13"/>
       <c r="H66" s="13"/>
       <c r="I66" s="13"/>
@@ -2448,325 +2539,532 @@
       <c r="K66" s="2"/>
       <c r="L66" s="2"/>
       <c r="M66" s="2"/>
+      <c r="N66" s="1" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="13"/>
-      <c r="B67" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="C67" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="D67" s="14"/>
-      <c r="E67" s="14"/>
-      <c r="F67" s="14"/>
-      <c r="G67" s="14"/>
-      <c r="H67" s="14"/>
-      <c r="I67" s="14"/>
-      <c r="J67" s="14"/>
-      <c r="K67" s="14"/>
-      <c r="L67" s="14"/>
-      <c r="M67" s="14"/>
-      <c r="N67" s="14"/>
-      <c r="O67" s="14"/>
-      <c r="P67" s="14"/>
-      <c r="Q67" s="15"/>
-      <c r="R67" s="15"/>
-      <c r="S67" s="15"/>
-      <c r="T67" s="15"/>
-    </row>
-    <row r="68" s="21" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2"/>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
+      <c r="D67" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F67" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="G67" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="H67" s="13"/>
+      <c r="I67" s="13"/>
+      <c r="J67" s="2"/>
+      <c r="K67" s="2"/>
+      <c r="L67" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M67" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="2"/>
       <c r="B68" s="2"/>
       <c r="C68" s="2"/>
-      <c r="D68" s="19"/>
-      <c r="E68" s="13"/>
-      <c r="F68" s="13"/>
-      <c r="G68" s="13"/>
+      <c r="D68" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E68" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="F68" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="G68" s="13" t="s">
+        <v>4</v>
+      </c>
       <c r="H68" s="13"/>
       <c r="I68" s="13"/>
       <c r="J68" s="2"/>
       <c r="K68" s="2"/>
-      <c r="L68" s="2"/>
-      <c r="M68" s="2"/>
-      <c r="N68" s="1"/>
-      <c r="O68" s="1"/>
-      <c r="P68" s="1"/>
-      <c r="Q68" s="1"/>
-      <c r="R68" s="1"/>
-      <c r="S68" s="1"/>
-      <c r="T68" s="1"/>
+      <c r="L68" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M68" s="2" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2"/>
       <c r="B69" s="2"/>
       <c r="C69" s="2"/>
-      <c r="D69" s="19"/>
-      <c r="E69" s="13"/>
-      <c r="F69" s="13"/>
-      <c r="G69" s="13"/>
+      <c r="D69" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F69" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="G69" s="13" t="s">
+        <v>4</v>
+      </c>
       <c r="H69" s="13"/>
       <c r="I69" s="13"/>
       <c r="J69" s="2"/>
       <c r="K69" s="2"/>
-      <c r="L69" s="2"/>
-      <c r="M69" s="2"/>
+      <c r="L69" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M69" s="2" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="21"/>
-      <c r="B70" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="C70" s="22" t="s">
-        <v>83</v>
-      </c>
-      <c r="D70" s="22"/>
-      <c r="E70" s="22"/>
-      <c r="F70" s="22"/>
-      <c r="G70" s="22"/>
-      <c r="H70" s="22"/>
-      <c r="I70" s="22"/>
-      <c r="J70" s="23"/>
-      <c r="K70" s="23"/>
-      <c r="L70" s="22"/>
-      <c r="M70" s="23"/>
-      <c r="N70" s="22"/>
-      <c r="O70" s="14"/>
-      <c r="P70" s="14"/>
-      <c r="Q70" s="21"/>
-      <c r="R70" s="21"/>
-      <c r="S70" s="21"/>
-      <c r="T70" s="21"/>
+      <c r="A70" s="2"/>
+      <c r="B70" s="2"/>
+      <c r="C70" s="2"/>
+      <c r="D70" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="E70" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F70" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="G70" s="13" t="s">
+        <v>4</v>
+      </c>
+      <c r="H70" s="13"/>
+      <c r="I70" s="13"/>
+      <c r="J70" s="2"/>
+      <c r="K70" s="2"/>
+      <c r="L70" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="M70" s="2" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="2"/>
-      <c r="B71" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="C71" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="J71" s="24" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="13"/>
+      <c r="B71" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="C71" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D71" s="14"/>
+      <c r="E71" s="14"/>
+      <c r="F71" s="14"/>
+      <c r="G71" s="14"/>
+      <c r="H71" s="14"/>
+      <c r="I71" s="14"/>
+      <c r="J71" s="14"/>
+      <c r="K71" s="14"/>
+      <c r="L71" s="14"/>
+      <c r="M71" s="14"/>
+      <c r="N71" s="14"/>
+      <c r="O71" s="14"/>
+      <c r="P71" s="14"/>
+      <c r="Q71" s="15"/>
+      <c r="R71" s="15"/>
+      <c r="S71" s="15"/>
+      <c r="T71" s="15"/>
+    </row>
+    <row r="72" s="15" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="2"/>
-      <c r="C72" s="24"/>
-      <c r="D72" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="J72" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="L72" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="N72" s="25"/>
+      <c r="B72" s="2"/>
+      <c r="C72" s="2"/>
+      <c r="D72" s="19"/>
+      <c r="E72" s="13"/>
+      <c r="F72" s="13"/>
+      <c r="G72" s="13"/>
+      <c r="H72" s="13"/>
+      <c r="I72" s="13"/>
+      <c r="J72" s="2"/>
+      <c r="K72" s="2"/>
+      <c r="L72" s="2"/>
+      <c r="M72" s="2"/>
+      <c r="N72" s="1"/>
+      <c r="O72" s="1"/>
+      <c r="P72" s="1"/>
+      <c r="Q72" s="1"/>
+      <c r="R72" s="1"/>
+      <c r="S72" s="1"/>
+      <c r="T72" s="1"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="2"/>
-      <c r="C73" s="24"/>
-      <c r="D73" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F73" s="1" t="s">
+      <c r="B73" s="2"/>
+      <c r="C73" s="2"/>
+      <c r="D73" s="19"/>
+      <c r="E73" s="13"/>
+      <c r="F73" s="13"/>
+      <c r="G73" s="13"/>
+      <c r="H73" s="13"/>
+      <c r="I73" s="13"/>
+      <c r="J73" s="2"/>
+      <c r="K73" s="2"/>
+      <c r="L73" s="2"/>
+      <c r="M73" s="2"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="13"/>
+      <c r="B74" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="J73" s="24" t="s">
-        <v>85</v>
-      </c>
-      <c r="L73" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="O73" s="2"/>
-      <c r="P73" s="2"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="2"/>
-      <c r="C74" s="24"/>
-      <c r="J74" s="24"/>
-      <c r="N74" s="25"/>
-      <c r="O74" s="2"/>
-      <c r="P74" s="2"/>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C74" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="D74" s="14"/>
+      <c r="E74" s="14"/>
+      <c r="F74" s="14"/>
+      <c r="G74" s="14"/>
+      <c r="H74" s="14"/>
+      <c r="I74" s="14"/>
+      <c r="J74" s="14"/>
+      <c r="K74" s="14"/>
+      <c r="L74" s="14"/>
+      <c r="M74" s="14"/>
+      <c r="N74" s="14"/>
+      <c r="O74" s="14"/>
+      <c r="P74" s="14"/>
+      <c r="Q74" s="15"/>
+      <c r="R74" s="15"/>
+      <c r="S74" s="15"/>
+      <c r="T74" s="15"/>
+    </row>
+    <row r="75" s="15" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="2"/>
-      <c r="C75" s="24"/>
-      <c r="J75" s="24"/>
-      <c r="O75" s="2"/>
-      <c r="P75" s="2"/>
+      <c r="B75" s="2"/>
+      <c r="C75" s="2"/>
+      <c r="D75" s="19"/>
+      <c r="E75" s="13"/>
+      <c r="F75" s="13"/>
+      <c r="G75" s="13"/>
+      <c r="H75" s="13"/>
+      <c r="I75" s="13"/>
+      <c r="J75" s="2"/>
+      <c r="K75" s="2"/>
+      <c r="L75" s="2"/>
+      <c r="M75" s="2"/>
+      <c r="N75" s="1"/>
+      <c r="O75" s="1"/>
+      <c r="P75" s="1"/>
+      <c r="Q75" s="1"/>
+      <c r="R75" s="1"/>
+      <c r="S75" s="1"/>
+      <c r="T75" s="1"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="2"/>
       <c r="B76" s="2"/>
       <c r="C76" s="2"/>
-      <c r="D76" s="2"/>
-      <c r="E76" s="2"/>
-      <c r="F76" s="2"/>
-      <c r="G76" s="2"/>
-      <c r="H76" s="2"/>
-      <c r="I76" s="2"/>
+      <c r="D76" s="19"/>
+      <c r="E76" s="13"/>
+      <c r="F76" s="13"/>
+      <c r="G76" s="13"/>
+      <c r="H76" s="13"/>
+      <c r="I76" s="13"/>
       <c r="J76" s="2"/>
       <c r="K76" s="2"/>
       <c r="L76" s="2"/>
       <c r="M76" s="2"/>
-      <c r="N76" s="2"/>
-      <c r="O76" s="2"/>
-      <c r="P76" s="2"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="2"/>
-      <c r="B77" s="2"/>
-      <c r="C77" s="2"/>
-      <c r="D77" s="2"/>
-      <c r="E77" s="2"/>
-      <c r="F77" s="2"/>
-      <c r="G77" s="2"/>
-      <c r="H77" s="2"/>
-      <c r="I77" s="2"/>
-      <c r="J77" s="2"/>
-      <c r="K77" s="2"/>
-      <c r="L77" s="2"/>
-      <c r="M77" s="2"/>
-      <c r="N77" s="2"/>
-      <c r="O77" s="2"/>
-      <c r="P77" s="2"/>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="13"/>
+      <c r="B77" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="C77" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="D77" s="14"/>
+      <c r="E77" s="14"/>
+      <c r="F77" s="14"/>
+      <c r="G77" s="14"/>
+      <c r="H77" s="14"/>
+      <c r="I77" s="14"/>
+      <c r="J77" s="14"/>
+      <c r="K77" s="14"/>
+      <c r="L77" s="14"/>
+      <c r="M77" s="14"/>
+      <c r="N77" s="14"/>
+      <c r="O77" s="14"/>
+      <c r="P77" s="14"/>
+      <c r="Q77" s="15"/>
+      <c r="R77" s="15"/>
+      <c r="S77" s="15"/>
+      <c r="T77" s="15"/>
+    </row>
+    <row r="78" s="21" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2"/>
       <c r="B78" s="2"/>
       <c r="C78" s="2"/>
-      <c r="D78" s="2"/>
-      <c r="E78" s="2"/>
-      <c r="F78" s="2"/>
-      <c r="G78" s="2"/>
-      <c r="H78" s="2"/>
-      <c r="I78" s="2"/>
+      <c r="D78" s="19"/>
+      <c r="E78" s="13"/>
+      <c r="F78" s="13"/>
+      <c r="G78" s="13"/>
+      <c r="H78" s="13"/>
+      <c r="I78" s="13"/>
       <c r="J78" s="2"/>
       <c r="K78" s="2"/>
       <c r="L78" s="2"/>
       <c r="M78" s="2"/>
-      <c r="N78" s="2"/>
-      <c r="O78" s="2"/>
-      <c r="P78" s="2"/>
+      <c r="N78" s="1"/>
+      <c r="O78" s="1"/>
+      <c r="P78" s="1"/>
+      <c r="Q78" s="1"/>
+      <c r="R78" s="1"/>
+      <c r="S78" s="1"/>
+      <c r="T78" s="1"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
-      <c r="D79" s="2"/>
-      <c r="E79" s="2"/>
-      <c r="F79" s="2"/>
-      <c r="G79" s="2"/>
-      <c r="H79" s="2"/>
-      <c r="I79" s="2"/>
+      <c r="D79" s="19"/>
+      <c r="E79" s="13"/>
+      <c r="F79" s="13"/>
+      <c r="G79" s="13"/>
+      <c r="H79" s="13"/>
+      <c r="I79" s="13"/>
       <c r="J79" s="2"/>
       <c r="K79" s="2"/>
       <c r="L79" s="2"/>
       <c r="M79" s="2"/>
-      <c r="N79" s="2"/>
-      <c r="O79" s="2"/>
-      <c r="P79" s="2"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="2"/>
-      <c r="B80" s="2"/>
-      <c r="C80" s="2"/>
-      <c r="D80" s="2"/>
-      <c r="E80" s="2"/>
-      <c r="F80" s="2"/>
-      <c r="G80" s="2"/>
-      <c r="H80" s="2"/>
-      <c r="I80" s="2"/>
-      <c r="J80" s="2"/>
-      <c r="K80" s="2"/>
-      <c r="L80" s="2"/>
-      <c r="M80" s="2"/>
-      <c r="N80" s="2"/>
-      <c r="O80" s="2"/>
-      <c r="P80" s="2"/>
+      <c r="A80" s="21"/>
+      <c r="B80" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="C80" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="D80" s="22"/>
+      <c r="E80" s="22"/>
+      <c r="F80" s="22"/>
+      <c r="G80" s="22"/>
+      <c r="H80" s="22"/>
+      <c r="I80" s="22"/>
+      <c r="J80" s="23"/>
+      <c r="K80" s="23"/>
+      <c r="L80" s="22"/>
+      <c r="M80" s="23"/>
+      <c r="N80" s="22"/>
+      <c r="O80" s="14"/>
+      <c r="P80" s="14"/>
+      <c r="Q80" s="21"/>
+      <c r="R80" s="21"/>
+      <c r="S80" s="21"/>
+      <c r="T80" s="21"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="2"/>
-      <c r="B81" s="2"/>
-      <c r="C81" s="2"/>
-      <c r="D81" s="2"/>
-      <c r="E81" s="2"/>
-      <c r="F81" s="2"/>
-      <c r="G81" s="2"/>
-      <c r="H81" s="2"/>
-      <c r="I81" s="2"/>
-      <c r="J81" s="2"/>
-      <c r="K81" s="2"/>
-      <c r="L81" s="2"/>
-      <c r="M81" s="2"/>
-      <c r="N81" s="2"/>
-      <c r="O81" s="2"/>
-      <c r="P81" s="2"/>
+      <c r="B81" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C81" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="J81" s="24" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="2"/>
-      <c r="B82" s="2"/>
-      <c r="C82" s="2"/>
-      <c r="D82" s="2"/>
-      <c r="E82" s="2"/>
-      <c r="F82" s="2"/>
-      <c r="G82" s="2"/>
-      <c r="H82" s="2"/>
-      <c r="I82" s="2"/>
-      <c r="J82" s="2"/>
-      <c r="K82" s="2"/>
-      <c r="L82" s="2"/>
-      <c r="M82" s="2"/>
-      <c r="N82" s="2"/>
-      <c r="O82" s="2"/>
-      <c r="P82" s="2"/>
+      <c r="C82" s="24"/>
+      <c r="D82" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="J82" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="L82" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="N82" s="25"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C83" s="2"/>
+      <c r="A83" s="2"/>
+      <c r="C83" s="24"/>
+      <c r="D83" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="J83" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="L83" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="O83" s="2"/>
+      <c r="P83" s="2"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C84" s="2"/>
+      <c r="A84" s="2"/>
+      <c r="C84" s="24"/>
+      <c r="J84" s="24"/>
+      <c r="N84" s="25"/>
+      <c r="O84" s="2"/>
+      <c r="P84" s="2"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C85" s="2"/>
+      <c r="A85" s="2"/>
+      <c r="C85" s="24"/>
+      <c r="J85" s="24"/>
+      <c r="O85" s="2"/>
+      <c r="P85" s="2"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="2"/>
+      <c r="B86" s="2"/>
       <c r="C86" s="2"/>
+      <c r="D86" s="2"/>
+      <c r="E86" s="2"/>
+      <c r="F86" s="2"/>
+      <c r="G86" s="2"/>
+      <c r="H86" s="2"/>
+      <c r="I86" s="2"/>
+      <c r="J86" s="2"/>
+      <c r="K86" s="2"/>
+      <c r="L86" s="2"/>
+      <c r="M86" s="2"/>
+      <c r="N86" s="2"/>
+      <c r="O86" s="2"/>
+      <c r="P86" s="2"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="2"/>
+      <c r="B87" s="2"/>
       <c r="C87" s="2"/>
+      <c r="D87" s="2"/>
+      <c r="E87" s="2"/>
+      <c r="F87" s="2"/>
+      <c r="G87" s="2"/>
+      <c r="H87" s="2"/>
+      <c r="I87" s="2"/>
+      <c r="J87" s="2"/>
+      <c r="K87" s="2"/>
+      <c r="L87" s="2"/>
+      <c r="M87" s="2"/>
+      <c r="N87" s="2"/>
+      <c r="O87" s="2"/>
+      <c r="P87" s="2"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="2"/>
+      <c r="B88" s="2"/>
       <c r="C88" s="2"/>
+      <c r="D88" s="2"/>
+      <c r="E88" s="2"/>
+      <c r="F88" s="2"/>
+      <c r="G88" s="2"/>
+      <c r="H88" s="2"/>
+      <c r="I88" s="2"/>
+      <c r="J88" s="2"/>
+      <c r="K88" s="2"/>
+      <c r="L88" s="2"/>
+      <c r="M88" s="2"/>
+      <c r="N88" s="2"/>
+      <c r="O88" s="2"/>
+      <c r="P88" s="2"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="2"/>
+      <c r="B89" s="2"/>
       <c r="C89" s="2"/>
+      <c r="D89" s="2"/>
+      <c r="E89" s="2"/>
+      <c r="F89" s="2"/>
+      <c r="G89" s="2"/>
+      <c r="H89" s="2"/>
+      <c r="I89" s="2"/>
+      <c r="J89" s="2"/>
+      <c r="K89" s="2"/>
+      <c r="L89" s="2"/>
+      <c r="M89" s="2"/>
+      <c r="N89" s="2"/>
+      <c r="O89" s="2"/>
+      <c r="P89" s="2"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="2"/>
+      <c r="B90" s="2"/>
       <c r="C90" s="2"/>
+      <c r="D90" s="2"/>
+      <c r="E90" s="2"/>
+      <c r="F90" s="2"/>
+      <c r="G90" s="2"/>
+      <c r="H90" s="2"/>
+      <c r="I90" s="2"/>
+      <c r="J90" s="2"/>
+      <c r="K90" s="2"/>
+      <c r="L90" s="2"/>
+      <c r="M90" s="2"/>
+      <c r="N90" s="2"/>
+      <c r="O90" s="2"/>
+      <c r="P90" s="2"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="2"/>
+      <c r="B91" s="2"/>
       <c r="C91" s="2"/>
+      <c r="D91" s="2"/>
+      <c r="E91" s="2"/>
+      <c r="F91" s="2"/>
+      <c r="G91" s="2"/>
+      <c r="H91" s="2"/>
+      <c r="I91" s="2"/>
+      <c r="J91" s="2"/>
+      <c r="K91" s="2"/>
+      <c r="L91" s="2"/>
+      <c r="M91" s="2"/>
+      <c r="N91" s="2"/>
+      <c r="O91" s="2"/>
+      <c r="P91" s="2"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="2"/>
+      <c r="B92" s="2"/>
       <c r="C92" s="2"/>
+      <c r="D92" s="2"/>
+      <c r="E92" s="2"/>
+      <c r="F92" s="2"/>
+      <c r="G92" s="2"/>
+      <c r="H92" s="2"/>
+      <c r="I92" s="2"/>
+      <c r="J92" s="2"/>
+      <c r="K92" s="2"/>
+      <c r="L92" s="2"/>
+      <c r="M92" s="2"/>
+      <c r="N92" s="2"/>
+      <c r="O92" s="2"/>
+      <c r="P92" s="2"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C93" s="2"/>
@@ -5258,33 +5556,63 @@
     <row r="922" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C922" s="2"/>
     </row>
+    <row r="923" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C923" s="2"/>
+    </row>
+    <row r="924" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C924" s="2"/>
+    </row>
+    <row r="925" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C925" s="2"/>
+    </row>
+    <row r="926" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C926" s="2"/>
+    </row>
+    <row r="927" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C927" s="2"/>
+    </row>
+    <row r="928" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C928" s="2"/>
+    </row>
+    <row r="929" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C929" s="2"/>
+    </row>
+    <row r="930" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C930" s="2"/>
+    </row>
+    <row r="931" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C931" s="2"/>
+    </row>
+    <row r="932" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C932" s="2"/>
+    </row>
   </sheetData>
-  <autoFilter ref="B10:P73"/>
+  <autoFilter ref="B10:P83"/>
   <mergeCells count="1">
     <mergeCell ref="F1:P6"/>
   </mergeCells>
   <dataValidations count="6">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C83:C922" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C93:C932" type="list">
       <formula1>"VARIABLE,ARRAY,RECORD"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="M12:M13 M15:M16 M18:M19 M21:M22 M24:M25 M27:M28 M30:M31 M33:M34 M36:M47 M49:M60 M62:M63 M65:M66 M68:M71" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="M12:M13 M15:M16 M18:M19 M21:M22 M24:M25 M27:M28 M30:M31 M33:M34 M36:M52 M54:M70 M72:M73 M75:M76 M78:M81" type="list">
       <formula1>"rx,tx"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="The Object code value shall be:&#10;VARIABLE&#10;RECORD&#10;ARRAY" errorStyle="stop" errorTitle="Object Code value" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C12:C13 C15:C16 C18:C19 C21:C22 C24:C25 C27:C28 C30:C31 C33:C34 C36:C47 C49:C60 C62:C63 C65:C66 C68:C82" type="list">
+    <dataValidation allowBlank="true" error="The Object code value shall be:&#10;VARIABLE&#10;RECORD&#10;ARRAY" errorStyle="stop" errorTitle="Object Code value" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="C12:C13 C15:C16 C18:C19 C21:C22 C24:C25 C27:C28 C30:C31 C33:C34 C36:C52 C54:C70 C72:C73 C75:C76 C78:C92" type="list">
       <formula1>"VARIABLE,ARRAY,RECORD"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="C11 C14 C17 C20 C23 C26 C29 C32 C35 C48 C61 C64 C67" type="none">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="true" sqref="C11 C14 C17 C20 C23 C26 C29 C32 C35 C53 C71 C74 C77" type="none">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="The value for the entry category shall be &#10;M : (mandatory)&#10;O : (optional) &#10;C : (conditional)" errorStyle="stop" errorTitle="Category" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="J12:J13 J15:J16 J18:J19 J21:J22 J24:J25 J27:J28 J30:J31 J33:J34 J36:J47 J49:J60 J62:J63 J65:J66 J68:J82" type="list">
+    <dataValidation allowBlank="true" error="The value for the entry category shall be &#10;M : (mandatory)&#10;O : (optional) &#10;C : (conditional)" errorStyle="stop" errorTitle="Category" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="J12:J13 J15:J16 J18:J19 J21:J22 J24:J25 J27:J28 J30:J31 J33:J34 J36:J52 J54:J70 J72:J73 J75:J76 J78:J92" type="list">
       <formula1>"M,O,C"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" error="The entry flag shall be&#10;B : (Backup)&#10;S : (Setting)" errorStyle="stop" errorTitle="Backup/Setting Flag" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="K12:K13 K15:K16 K18:K19 K21:K22 K24:K25 K27:K28 K30:K31 K33:K34 K36:K47 K49:K60 K62:K63 K65:K66 K68:K82" type="list">
+    <dataValidation allowBlank="true" error="The entry flag shall be&#10;B : (Backup)&#10;S : (Setting)" errorStyle="stop" errorTitle="Backup/Setting Flag" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="K12:K13 K15:K16 K18:K19 K21:K22 K24:K25 K27:K28 K30:K31 K33:K34 K36:K52 K54:K70 K72:K73 K75:K76 K78:K92" type="list">
       <formula1>"B,S"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>